<commit_message>
fix set_loc data type
</commit_message>
<xml_diff>
--- a/data/split/test.xlsx
+++ b/data/split/test.xlsx
@@ -550,8 +550,10 @@
       <c r="L2" t="n">
         <v>4</v>
       </c>
-      <c r="M2" t="n">
-        <v>4</v>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N2" t="n">
         <v>2</v>
@@ -617,8 +619,10 @@
       <c r="L3" t="n">
         <v>5</v>
       </c>
-      <c r="M3" t="n">
-        <v>1</v>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N3" t="n">
         <v>2</v>
@@ -684,8 +688,10 @@
       <c r="L4" t="n">
         <v>5</v>
       </c>
-      <c r="M4" t="n">
-        <v>4</v>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N4" t="n">
         <v>1</v>
@@ -751,8 +757,10 @@
       <c r="L5" t="n">
         <v>5</v>
       </c>
-      <c r="M5" t="n">
-        <v>4</v>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N5" t="n">
         <v>1</v>
@@ -818,8 +826,10 @@
       <c r="L6" t="n">
         <v>3</v>
       </c>
-      <c r="M6" t="n">
-        <v>4</v>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N6" t="n">
         <v>2</v>
@@ -885,8 +895,10 @@
       <c r="L7" t="n">
         <v>2</v>
       </c>
-      <c r="M7" t="n">
-        <v>5</v>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N7" t="n">
         <v>2</v>
@@ -952,8 +964,10 @@
       <c r="L8" t="n">
         <v>5</v>
       </c>
-      <c r="M8" t="n">
-        <v>1</v>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N8" t="n">
         <v>2</v>
@@ -1019,8 +1033,10 @@
       <c r="L9" t="n">
         <v>2</v>
       </c>
-      <c r="M9" t="n">
-        <v>3</v>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="N9" t="n">
         <v>2</v>
@@ -1086,8 +1102,10 @@
       <c r="L10" t="n">
         <v>4</v>
       </c>
-      <c r="M10" t="n">
-        <v>4</v>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N10" t="n">
         <v>2</v>
@@ -1153,8 +1171,10 @@
       <c r="L11" t="n">
         <v>4</v>
       </c>
-      <c r="M11" t="n">
-        <v>1</v>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N11" t="n">
         <v>1</v>
@@ -1358,8 +1378,10 @@
       <c r="L14" t="n">
         <v>4</v>
       </c>
-      <c r="M14" t="n">
-        <v>4</v>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N14" t="n">
         <v>2</v>
@@ -1563,8 +1585,10 @@
       <c r="L17" t="n">
         <v>3</v>
       </c>
-      <c r="M17" t="n">
-        <v>4</v>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N17" t="n">
         <v>1</v>
@@ -1768,8 +1792,10 @@
       <c r="L20" t="n">
         <v>4</v>
       </c>
-      <c r="M20" t="n">
-        <v>1</v>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N20" t="n">
         <v>1</v>
@@ -1835,8 +1861,10 @@
       <c r="L21" t="n">
         <v>2</v>
       </c>
-      <c r="M21" t="n">
-        <v>4</v>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N21" t="n">
         <v>3</v>
@@ -1971,8 +1999,10 @@
       <c r="L23" t="n">
         <v>4</v>
       </c>
-      <c r="M23" t="n">
-        <v>4</v>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N23" t="n">
         <v>2</v>
@@ -2038,8 +2068,10 @@
       <c r="L24" t="n">
         <v>5</v>
       </c>
-      <c r="M24" t="n">
-        <v>4</v>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N24" t="n">
         <v>2</v>
@@ -2174,8 +2206,10 @@
       <c r="L26" t="n">
         <v>4</v>
       </c>
-      <c r="M26" t="n">
-        <v>4</v>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N26" t="n">
         <v>2</v>
@@ -2379,8 +2413,10 @@
       <c r="L29" t="n">
         <v>4</v>
       </c>
-      <c r="M29" t="n">
-        <v>4</v>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N29" t="n">
         <v>2</v>
@@ -2446,8 +2482,10 @@
       <c r="L30" t="n">
         <v>4</v>
       </c>
-      <c r="M30" t="n">
-        <v>4</v>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N30" t="n">
         <v>2</v>
@@ -2513,8 +2551,10 @@
       <c r="L31" t="n">
         <v>4</v>
       </c>
-      <c r="M31" t="n">
-        <v>4</v>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N31" t="n">
         <v>2</v>
@@ -2718,8 +2758,10 @@
       <c r="L34" t="n">
         <v>5</v>
       </c>
-      <c r="M34" t="n">
-        <v>4</v>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N34" t="n">
         <v>1</v>
@@ -2785,8 +2827,10 @@
       <c r="L35" t="n">
         <v>4</v>
       </c>
-      <c r="M35" t="n">
-        <v>5</v>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N35" t="n">
         <v>2</v>
@@ -2852,8 +2896,10 @@
       <c r="L36" t="n">
         <v>3</v>
       </c>
-      <c r="M36" t="n">
-        <v>4</v>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N36" t="n">
         <v>2</v>
@@ -2988,8 +3034,10 @@
       <c r="L38" t="n">
         <v>4</v>
       </c>
-      <c r="M38" t="n">
-        <v>3</v>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="N38" t="n">
         <v>2</v>
@@ -3193,8 +3241,10 @@
       <c r="L41" t="n">
         <v>5</v>
       </c>
-      <c r="M41" t="n">
-        <v>1</v>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N41" t="n">
         <v>0</v>
@@ -3329,8 +3379,10 @@
       <c r="L43" t="n">
         <v>4</v>
       </c>
-      <c r="M43" t="n">
-        <v>4</v>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N43" t="n">
         <v>2</v>
@@ -3396,8 +3448,10 @@
       <c r="L44" t="n">
         <v>4</v>
       </c>
-      <c r="M44" t="n">
-        <v>4</v>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N44" t="n">
         <v>2</v>
@@ -3463,8 +3517,10 @@
       <c r="L45" t="n">
         <v>4</v>
       </c>
-      <c r="M45" t="n">
-        <v>4</v>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N45" t="n">
         <v>2</v>
@@ -3530,8 +3586,10 @@
       <c r="L46" t="n">
         <v>5</v>
       </c>
-      <c r="M46" t="n">
-        <v>4</v>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N46" t="n">
         <v>2</v>
@@ -3597,8 +3655,10 @@
       <c r="L47" t="n">
         <v>3</v>
       </c>
-      <c r="M47" t="n">
-        <v>4</v>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N47" t="n">
         <v>2</v>
@@ -3664,8 +3724,10 @@
       <c r="L48" t="n">
         <v>4</v>
       </c>
-      <c r="M48" t="n">
-        <v>4</v>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N48" t="n">
         <v>2</v>
@@ -3869,8 +3931,10 @@
       <c r="L51" t="n">
         <v>5</v>
       </c>
-      <c r="M51" t="n">
-        <v>1</v>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N51" t="n">
         <v>2</v>
@@ -3936,8 +4000,10 @@
       <c r="L52" t="n">
         <v>4</v>
       </c>
-      <c r="M52" t="n">
-        <v>4</v>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N52" t="n">
         <v>2</v>
@@ -4072,8 +4138,10 @@
       <c r="L54" t="n">
         <v>5</v>
       </c>
-      <c r="M54" t="n">
-        <v>2</v>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="N54" t="n">
         <v>2</v>
@@ -4208,8 +4276,10 @@
       <c r="L56" t="n">
         <v>4</v>
       </c>
-      <c r="M56" t="n">
-        <v>4</v>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N56" t="n">
         <v>2</v>
@@ -4275,8 +4345,10 @@
       <c r="L57" t="n">
         <v>4</v>
       </c>
-      <c r="M57" t="n">
-        <v>1</v>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N57" t="n">
         <v>1</v>
@@ -4342,8 +4414,10 @@
       <c r="L58" t="n">
         <v>5</v>
       </c>
-      <c r="M58" t="n">
-        <v>1</v>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N58" t="n">
         <v>1</v>
@@ -4409,8 +4483,10 @@
       <c r="L59" t="n">
         <v>3</v>
       </c>
-      <c r="M59" t="n">
-        <v>5</v>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N59" t="n">
         <v>1</v>
@@ -4545,8 +4621,10 @@
       <c r="L61" t="n">
         <v>5</v>
       </c>
-      <c r="M61" t="n">
-        <v>1</v>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N61" t="n">
         <v>1</v>
@@ -4681,8 +4759,10 @@
       <c r="L63" t="n">
         <v>4</v>
       </c>
-      <c r="M63" t="n">
-        <v>5</v>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N63" t="n">
         <v>2</v>
@@ -4748,8 +4828,10 @@
       <c r="L64" t="n">
         <v>2</v>
       </c>
-      <c r="M64" t="n">
-        <v>5</v>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N64" t="n">
         <v>2</v>
@@ -4815,8 +4897,10 @@
       <c r="L65" t="n">
         <v>4</v>
       </c>
-      <c r="M65" t="n">
-        <v>5</v>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N65" t="n">
         <v>2</v>
@@ -4951,8 +5035,10 @@
       <c r="L67" t="n">
         <v>4</v>
       </c>
-      <c r="M67" t="n">
-        <v>5</v>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N67" t="n">
         <v>2</v>
@@ -5018,8 +5104,10 @@
       <c r="L68" t="n">
         <v>2</v>
       </c>
-      <c r="M68" t="n">
-        <v>4</v>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N68" t="n">
         <v>3</v>
@@ -5085,8 +5173,10 @@
       <c r="L69" t="n">
         <v>2</v>
       </c>
-      <c r="M69" t="n">
-        <v>5</v>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N69" t="n">
         <v>3</v>
@@ -5152,8 +5242,10 @@
       <c r="L70" t="n">
         <v>4</v>
       </c>
-      <c r="M70" t="n">
-        <v>4</v>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N70" t="n">
         <v>2</v>
@@ -5219,8 +5311,10 @@
       <c r="L71" t="n">
         <v>4</v>
       </c>
-      <c r="M71" t="n">
-        <v>4</v>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N71" t="n">
         <v>2</v>
@@ -5286,8 +5380,10 @@
       <c r="L72" t="n">
         <v>5</v>
       </c>
-      <c r="M72" t="n">
-        <v>1</v>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N72" t="n">
         <v>2</v>
@@ -5422,8 +5518,10 @@
       <c r="L74" t="n">
         <v>2</v>
       </c>
-      <c r="M74" t="n">
-        <v>3</v>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="N74" t="n">
         <v>2</v>
@@ -5489,8 +5587,10 @@
       <c r="L75" t="n">
         <v>4</v>
       </c>
-      <c r="M75" t="n">
-        <v>2</v>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="N75" t="n">
         <v>1</v>
@@ -5694,8 +5794,10 @@
       <c r="L78" t="n">
         <v>2</v>
       </c>
-      <c r="M78" t="n">
-        <v>4</v>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N78" t="n">
         <v>2</v>
@@ -5761,8 +5863,10 @@
       <c r="L79" t="n">
         <v>4</v>
       </c>
-      <c r="M79" t="n">
-        <v>4</v>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N79" t="n">
         <v>2</v>
@@ -5828,8 +5932,10 @@
       <c r="L80" t="n">
         <v>4</v>
       </c>
-      <c r="M80" t="n">
-        <v>5</v>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N80" t="n">
         <v>2</v>
@@ -5895,8 +6001,10 @@
       <c r="L81" t="n">
         <v>2</v>
       </c>
-      <c r="M81" t="n">
-        <v>4</v>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N81" t="n">
         <v>2</v>
@@ -5962,8 +6070,10 @@
       <c r="L82" t="n">
         <v>5</v>
       </c>
-      <c r="M82" t="n">
-        <v>4</v>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N82" t="n">
         <v>2</v>
@@ -6029,8 +6139,10 @@
       <c r="L83" t="n">
         <v>4</v>
       </c>
-      <c r="M83" t="n">
-        <v>1</v>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N83" t="n">
         <v>1</v>
@@ -6096,8 +6208,10 @@
       <c r="L84" t="n">
         <v>4</v>
       </c>
-      <c r="M84" t="n">
-        <v>4</v>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N84" t="n">
         <v>1</v>
@@ -6232,8 +6346,10 @@
       <c r="L86" t="n">
         <v>2</v>
       </c>
-      <c r="M86" t="n">
-        <v>4</v>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N86" t="n">
         <v>2</v>
@@ -6299,8 +6415,10 @@
       <c r="L87" t="n">
         <v>2</v>
       </c>
-      <c r="M87" t="n">
-        <v>4</v>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N87" t="n">
         <v>3</v>
@@ -6366,8 +6484,10 @@
       <c r="L88" t="n">
         <v>4</v>
       </c>
-      <c r="M88" t="n">
-        <v>4</v>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N88" t="n">
         <v>2</v>
@@ -6502,8 +6622,10 @@
       <c r="L90" t="n">
         <v>4</v>
       </c>
-      <c r="M90" t="n">
-        <v>4</v>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N90" t="n">
         <v>2</v>
@@ -6569,8 +6691,10 @@
       <c r="L91" t="n">
         <v>3</v>
       </c>
-      <c r="M91" t="n">
-        <v>4</v>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N91" t="n">
         <v>2</v>
@@ -6774,8 +6898,10 @@
       <c r="L94" t="n">
         <v>4</v>
       </c>
-      <c r="M94" t="n">
-        <v>4</v>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N94" t="n">
         <v>2</v>
@@ -6841,8 +6967,10 @@
       <c r="L95" t="n">
         <v>5</v>
       </c>
-      <c r="M95" t="n">
-        <v>4</v>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N95" t="n">
         <v>2</v>
@@ -6908,8 +7036,10 @@
       <c r="L96" t="n">
         <v>3</v>
       </c>
-      <c r="M96" t="n">
-        <v>5</v>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N96" t="n">
         <v>2</v>
@@ -7044,8 +7174,10 @@
       <c r="L98" t="n">
         <v>4</v>
       </c>
-      <c r="M98" t="n">
-        <v>4</v>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N98" t="n">
         <v>2</v>
@@ -7111,8 +7243,10 @@
       <c r="L99" t="n">
         <v>5</v>
       </c>
-      <c r="M99" t="n">
-        <v>5</v>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N99" t="n">
         <v>2</v>
@@ -7178,8 +7312,10 @@
       <c r="L100" t="n">
         <v>4</v>
       </c>
-      <c r="M100" t="n">
-        <v>5</v>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N100" t="n">
         <v>2</v>
@@ -7245,8 +7381,10 @@
       <c r="L101" t="n">
         <v>5</v>
       </c>
-      <c r="M101" t="n">
-        <v>3</v>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="N101" t="n">
         <v>2</v>
@@ -7450,8 +7588,10 @@
       <c r="L104" t="n">
         <v>5</v>
       </c>
-      <c r="M104" t="n">
-        <v>5</v>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N104" t="n">
         <v>2</v>
@@ -7517,8 +7657,10 @@
       <c r="L105" t="n">
         <v>4</v>
       </c>
-      <c r="M105" t="n">
-        <v>4</v>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N105" t="n">
         <v>2</v>
@@ -7584,8 +7726,10 @@
       <c r="L106" t="n">
         <v>4</v>
       </c>
-      <c r="M106" t="n">
-        <v>4</v>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N106" t="n">
         <v>2</v>
@@ -7651,8 +7795,10 @@
       <c r="L107" t="n">
         <v>4</v>
       </c>
-      <c r="M107" t="n">
-        <v>4</v>
+      <c r="M107" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N107" t="n">
         <v>2</v>
@@ -7718,8 +7864,10 @@
       <c r="L108" t="n">
         <v>4</v>
       </c>
-      <c r="M108" t="n">
-        <v>4</v>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N108" t="n">
         <v>2</v>
@@ -7785,8 +7933,10 @@
       <c r="L109" t="n">
         <v>2</v>
       </c>
-      <c r="M109" t="n">
-        <v>4</v>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N109" t="n">
         <v>2</v>
@@ -7921,8 +8071,10 @@
       <c r="L111" t="n">
         <v>5</v>
       </c>
-      <c r="M111" t="n">
-        <v>4</v>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N111" t="n">
         <v>2</v>
@@ -8057,8 +8209,10 @@
       <c r="L113" t="n">
         <v>4</v>
       </c>
-      <c r="M113" t="n">
-        <v>4</v>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N113" t="n">
         <v>2</v>
@@ -8124,8 +8278,10 @@
       <c r="L114" t="n">
         <v>3</v>
       </c>
-      <c r="M114" t="n">
-        <v>4</v>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N114" t="n">
         <v>2</v>
@@ -8191,8 +8347,10 @@
       <c r="L115" t="n">
         <v>2</v>
       </c>
-      <c r="M115" t="n">
-        <v>5</v>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N115" t="n">
         <v>2</v>
@@ -8258,8 +8416,10 @@
       <c r="L116" t="n">
         <v>1</v>
       </c>
-      <c r="M116" t="n">
-        <v>5</v>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N116" t="n">
         <v>2</v>
@@ -8394,8 +8554,10 @@
       <c r="L118" t="n">
         <v>5</v>
       </c>
-      <c r="M118" t="n">
-        <v>4</v>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N118" t="n">
         <v>2</v>
@@ -8461,8 +8623,10 @@
       <c r="L119" t="n">
         <v>2</v>
       </c>
-      <c r="M119" t="n">
-        <v>4</v>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N119" t="n">
         <v>2</v>
@@ -8597,8 +8761,10 @@
       <c r="L121" t="n">
         <v>5</v>
       </c>
-      <c r="M121" t="n">
-        <v>4</v>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N121" t="n">
         <v>2</v>
@@ -8664,8 +8830,10 @@
       <c r="L122" t="n">
         <v>4</v>
       </c>
-      <c r="M122" t="n">
-        <v>5</v>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N122" t="n">
         <v>1</v>
@@ -8731,8 +8899,10 @@
       <c r="L123" t="n">
         <v>3</v>
       </c>
-      <c r="M123" t="n">
-        <v>4</v>
+      <c r="M123" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N123" t="n">
         <v>2</v>
@@ -8936,8 +9106,10 @@
       <c r="L126" t="n">
         <v>5</v>
       </c>
-      <c r="M126" t="n">
-        <v>4</v>
+      <c r="M126" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N126" t="n">
         <v>2</v>
@@ -9003,8 +9175,10 @@
       <c r="L127" t="n">
         <v>3</v>
       </c>
-      <c r="M127" t="n">
-        <v>1</v>
+      <c r="M127" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N127" t="n">
         <v>0</v>
@@ -9139,8 +9313,10 @@
       <c r="L129" t="n">
         <v>2</v>
       </c>
-      <c r="M129" t="n">
-        <v>4</v>
+      <c r="M129" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N129" t="n">
         <v>2</v>
@@ -9206,8 +9382,10 @@
       <c r="L130" t="n">
         <v>5</v>
       </c>
-      <c r="M130" t="n">
-        <v>4</v>
+      <c r="M130" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N130" t="n">
         <v>2</v>
@@ -9342,8 +9520,10 @@
       <c r="L132" t="n">
         <v>4</v>
       </c>
-      <c r="M132" t="n">
-        <v>4</v>
+      <c r="M132" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N132" t="n">
         <v>2</v>
@@ -9409,8 +9589,10 @@
       <c r="L133" t="n">
         <v>5</v>
       </c>
-      <c r="M133" t="n">
-        <v>1</v>
+      <c r="M133" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N133" t="n">
         <v>2</v>
@@ -9614,8 +9796,10 @@
       <c r="L136" t="n">
         <v>3</v>
       </c>
-      <c r="M136" t="n">
-        <v>1</v>
+      <c r="M136" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N136" t="n">
         <v>2</v>
@@ -9681,8 +9865,10 @@
       <c r="L137" t="n">
         <v>4</v>
       </c>
-      <c r="M137" t="n">
-        <v>4</v>
+      <c r="M137" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N137" t="n">
         <v>2</v>
@@ -9748,8 +9934,10 @@
       <c r="L138" t="n">
         <v>4</v>
       </c>
-      <c r="M138" t="n">
-        <v>3</v>
+      <c r="M138" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="N138" t="n">
         <v>2</v>
@@ -9815,8 +10003,10 @@
       <c r="L139" t="n">
         <v>2</v>
       </c>
-      <c r="M139" t="n">
-        <v>4</v>
+      <c r="M139" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N139" t="n">
         <v>2</v>
@@ -9951,8 +10141,10 @@
       <c r="L141" t="n">
         <v>5</v>
       </c>
-      <c r="M141" t="n">
-        <v>4</v>
+      <c r="M141" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N141" t="n">
         <v>1</v>
@@ -10018,8 +10210,10 @@
       <c r="L142" t="n">
         <v>5</v>
       </c>
-      <c r="M142" t="n">
-        <v>4</v>
+      <c r="M142" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N142" t="n">
         <v>2</v>
@@ -10085,8 +10279,10 @@
       <c r="L143" t="n">
         <v>4</v>
       </c>
-      <c r="M143" t="n">
-        <v>1</v>
+      <c r="M143" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N143" t="n">
         <v>0</v>
@@ -10359,8 +10555,10 @@
       <c r="L147" t="n">
         <v>5</v>
       </c>
-      <c r="M147" t="n">
-        <v>4</v>
+      <c r="M147" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N147" t="n">
         <v>1</v>
@@ -10426,8 +10624,10 @@
       <c r="L148" t="n">
         <v>4</v>
       </c>
-      <c r="M148" t="n">
-        <v>1</v>
+      <c r="M148" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N148" t="n">
         <v>2</v>
@@ -10562,8 +10762,10 @@
       <c r="L150" t="n">
         <v>3</v>
       </c>
-      <c r="M150" t="n">
-        <v>3</v>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="N150" t="n">
         <v>2</v>
@@ -10629,8 +10831,10 @@
       <c r="L151" t="n">
         <v>5</v>
       </c>
-      <c r="M151" t="n">
-        <v>4</v>
+      <c r="M151" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N151" t="n">
         <v>1</v>
@@ -10834,8 +11038,10 @@
       <c r="L154" t="n">
         <v>4</v>
       </c>
-      <c r="M154" t="n">
-        <v>4</v>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N154" t="n">
         <v>2</v>
@@ -10901,8 +11107,10 @@
       <c r="L155" t="n">
         <v>4</v>
       </c>
-      <c r="M155" t="n">
-        <v>2</v>
+      <c r="M155" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="N155" t="n">
         <v>2</v>
@@ -11037,8 +11245,10 @@
       <c r="L157" t="n">
         <v>5</v>
       </c>
-      <c r="M157" t="n">
-        <v>4</v>
+      <c r="M157" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N157" t="n">
         <v>2</v>
@@ -11104,8 +11314,10 @@
       <c r="L158" t="n">
         <v>4</v>
       </c>
-      <c r="M158" t="n">
-        <v>5</v>
+      <c r="M158" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N158" t="n">
         <v>2</v>
@@ -11171,8 +11383,10 @@
       <c r="L159" t="n">
         <v>3</v>
       </c>
-      <c r="M159" t="n">
-        <v>4</v>
+      <c r="M159" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N159" t="n">
         <v>2</v>
@@ -11376,8 +11590,10 @@
       <c r="L162" t="n">
         <v>5</v>
       </c>
-      <c r="M162" t="n">
-        <v>1</v>
+      <c r="M162" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N162" t="n">
         <v>1</v>
@@ -11443,8 +11659,10 @@
       <c r="L163" t="n">
         <v>4</v>
       </c>
-      <c r="M163" t="n">
-        <v>4</v>
+      <c r="M163" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N163" t="n">
         <v>2</v>
@@ -11510,8 +11728,10 @@
       <c r="L164" t="n">
         <v>4</v>
       </c>
-      <c r="M164" t="n">
-        <v>4</v>
+      <c r="M164" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N164" t="n">
         <v>2</v>
@@ -11577,8 +11797,10 @@
       <c r="L165" t="n">
         <v>2</v>
       </c>
-      <c r="M165" t="n">
-        <v>4</v>
+      <c r="M165" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N165" t="n">
         <v>2</v>
@@ -11644,8 +11866,10 @@
       <c r="L166" t="n">
         <v>5</v>
       </c>
-      <c r="M166" t="n">
-        <v>4</v>
+      <c r="M166" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N166" t="n">
         <v>1</v>
@@ -11711,8 +11935,10 @@
       <c r="L167" t="n">
         <v>2</v>
       </c>
-      <c r="M167" t="n">
-        <v>4</v>
+      <c r="M167" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N167" t="n">
         <v>0</v>
@@ -11778,8 +12004,10 @@
       <c r="L168" t="n">
         <v>5</v>
       </c>
-      <c r="M168" t="n">
-        <v>1</v>
+      <c r="M168" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N168" t="n">
         <v>2</v>
@@ -11914,8 +12142,10 @@
       <c r="L170" t="n">
         <v>4</v>
       </c>
-      <c r="M170" t="n">
-        <v>4</v>
+      <c r="M170" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N170" t="n">
         <v>2</v>
@@ -11981,8 +12211,10 @@
       <c r="L171" t="n">
         <v>4</v>
       </c>
-      <c r="M171" t="n">
-        <v>4</v>
+      <c r="M171" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N171" t="n">
         <v>2</v>
@@ -12048,8 +12280,10 @@
       <c r="L172" t="n">
         <v>4</v>
       </c>
-      <c r="M172" t="n">
-        <v>4</v>
+      <c r="M172" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N172" t="n">
         <v>0</v>
@@ -12184,8 +12418,10 @@
       <c r="L174" t="n">
         <v>4</v>
       </c>
-      <c r="M174" t="n">
-        <v>4</v>
+      <c r="M174" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N174" t="n">
         <v>2</v>
@@ -12458,8 +12694,10 @@
       <c r="L178" t="n">
         <v>2</v>
       </c>
-      <c r="M178" t="n">
-        <v>5</v>
+      <c r="M178" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N178" t="n">
         <v>2</v>
@@ -12525,8 +12763,10 @@
       <c r="L179" t="n">
         <v>4</v>
       </c>
-      <c r="M179" t="n">
-        <v>4</v>
+      <c r="M179" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N179" t="n">
         <v>2</v>
@@ -12661,8 +12901,10 @@
       <c r="L181" t="n">
         <v>4</v>
       </c>
-      <c r="M181" t="n">
-        <v>5</v>
+      <c r="M181" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N181" t="n">
         <v>2</v>
@@ -12728,8 +12970,10 @@
       <c r="L182" t="n">
         <v>5</v>
       </c>
-      <c r="M182" t="n">
-        <v>5</v>
+      <c r="M182" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N182" t="n">
         <v>2</v>
@@ -12795,8 +13039,10 @@
       <c r="L183" t="n">
         <v>3</v>
       </c>
-      <c r="M183" t="n">
-        <v>4</v>
+      <c r="M183" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N183" t="n">
         <v>2</v>
@@ -12862,8 +13108,10 @@
       <c r="L184" t="n">
         <v>4</v>
       </c>
-      <c r="M184" t="n">
-        <v>5</v>
+      <c r="M184" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N184" t="n">
         <v>1</v>
@@ -13136,8 +13384,10 @@
       <c r="L188" t="n">
         <v>2</v>
       </c>
-      <c r="M188" t="n">
-        <v>4</v>
+      <c r="M188" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N188" t="n">
         <v>3</v>
@@ -13272,8 +13522,10 @@
       <c r="L190" t="n">
         <v>2</v>
       </c>
-      <c r="M190" t="n">
-        <v>4</v>
+      <c r="M190" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N190" t="n">
         <v>3</v>
@@ -13339,8 +13591,10 @@
       <c r="L191" t="n">
         <v>3</v>
       </c>
-      <c r="M191" t="n">
-        <v>4</v>
+      <c r="M191" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N191" t="n">
         <v>2</v>
@@ -13406,8 +13660,10 @@
       <c r="L192" t="n">
         <v>5</v>
       </c>
-      <c r="M192" t="n">
-        <v>1</v>
+      <c r="M192" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N192" t="n">
         <v>2</v>
@@ -13473,8 +13729,10 @@
       <c r="L193" t="n">
         <v>4</v>
       </c>
-      <c r="M193" t="n">
-        <v>4</v>
+      <c r="M193" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N193" t="n">
         <v>2</v>
@@ -13609,8 +13867,10 @@
       <c r="L195" t="n">
         <v>3</v>
       </c>
-      <c r="M195" t="n">
-        <v>4</v>
+      <c r="M195" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N195" t="n">
         <v>2</v>
@@ -13676,8 +13936,10 @@
       <c r="L196" t="n">
         <v>5</v>
       </c>
-      <c r="M196" t="n">
-        <v>4</v>
+      <c r="M196" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N196" t="n">
         <v>2</v>
@@ -13812,8 +14074,10 @@
       <c r="L198" t="n">
         <v>2</v>
       </c>
-      <c r="M198" t="n">
-        <v>4</v>
+      <c r="M198" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N198" t="n">
         <v>2</v>
@@ -13948,8 +14212,10 @@
       <c r="L200" t="n">
         <v>4</v>
       </c>
-      <c r="M200" t="n">
-        <v>4</v>
+      <c r="M200" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N200" t="n">
         <v>2</v>
@@ -14015,8 +14281,10 @@
       <c r="L201" t="n">
         <v>4</v>
       </c>
-      <c r="M201" t="n">
-        <v>4</v>
+      <c r="M201" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N201" t="n">
         <v>2</v>
@@ -14082,8 +14350,10 @@
       <c r="L202" t="n">
         <v>2</v>
       </c>
-      <c r="M202" t="n">
-        <v>4</v>
+      <c r="M202" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N202" t="n">
         <v>1</v>
@@ -14149,8 +14419,10 @@
       <c r="L203" t="n">
         <v>5</v>
       </c>
-      <c r="M203" t="n">
-        <v>1</v>
+      <c r="M203" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N203" t="n">
         <v>1</v>
@@ -14285,8 +14557,10 @@
       <c r="L205" t="n">
         <v>3</v>
       </c>
-      <c r="M205" t="n">
-        <v>4</v>
+      <c r="M205" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N205" t="n">
         <v>2</v>
@@ -14421,8 +14695,10 @@
       <c r="L207" t="n">
         <v>4</v>
       </c>
-      <c r="M207" t="n">
-        <v>4</v>
+      <c r="M207" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N207" t="n">
         <v>2</v>
@@ -14557,8 +14833,10 @@
       <c r="L209" t="n">
         <v>2</v>
       </c>
-      <c r="M209" t="n">
-        <v>4</v>
+      <c r="M209" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N209" t="n">
         <v>3</v>
@@ -14693,8 +14971,10 @@
       <c r="L211" t="n">
         <v>4</v>
       </c>
-      <c r="M211" t="n">
-        <v>4</v>
+      <c r="M211" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N211" t="n">
         <v>2</v>
@@ -14760,8 +15040,10 @@
       <c r="L212" t="n">
         <v>2</v>
       </c>
-      <c r="M212" t="n">
-        <v>4</v>
+      <c r="M212" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N212" t="n">
         <v>2</v>
@@ -14827,8 +15109,10 @@
       <c r="L213" t="n">
         <v>4</v>
       </c>
-      <c r="M213" t="n">
-        <v>4</v>
+      <c r="M213" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N213" t="n">
         <v>2</v>
@@ -14894,8 +15178,10 @@
       <c r="L214" t="n">
         <v>4</v>
       </c>
-      <c r="M214" t="n">
-        <v>5</v>
+      <c r="M214" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N214" t="n">
         <v>2</v>
@@ -15099,8 +15385,10 @@
       <c r="L217" t="n">
         <v>5</v>
       </c>
-      <c r="M217" t="n">
-        <v>4</v>
+      <c r="M217" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N217" t="n">
         <v>2</v>
@@ -15235,8 +15523,10 @@
       <c r="L219" t="n">
         <v>5</v>
       </c>
-      <c r="M219" t="n">
-        <v>5</v>
+      <c r="M219" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N219" t="n">
         <v>2</v>
@@ -15302,8 +15592,10 @@
       <c r="L220" t="n">
         <v>5</v>
       </c>
-      <c r="M220" t="n">
-        <v>4</v>
+      <c r="M220" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N220" t="n">
         <v>2</v>
@@ -15438,8 +15730,10 @@
       <c r="L222" t="n">
         <v>2</v>
       </c>
-      <c r="M222" t="n">
-        <v>4</v>
+      <c r="M222" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N222" t="n">
         <v>3</v>
@@ -15574,8 +15868,10 @@
       <c r="L224" t="n">
         <v>3</v>
       </c>
-      <c r="M224" t="n">
-        <v>5</v>
+      <c r="M224" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N224" t="n">
         <v>2</v>
@@ -15641,8 +15937,10 @@
       <c r="L225" t="n">
         <v>4</v>
       </c>
-      <c r="M225" t="n">
-        <v>4</v>
+      <c r="M225" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N225" t="n">
         <v>2</v>
@@ -15777,8 +16075,10 @@
       <c r="L227" t="n">
         <v>4</v>
       </c>
-      <c r="M227" t="n">
-        <v>4</v>
+      <c r="M227" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N227" t="n">
         <v>2</v>
@@ -15844,8 +16144,10 @@
       <c r="L228" t="n">
         <v>4</v>
       </c>
-      <c r="M228" t="n">
-        <v>4</v>
+      <c r="M228" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N228" t="n">
         <v>2</v>
@@ -15911,8 +16213,10 @@
       <c r="L229" t="n">
         <v>3</v>
       </c>
-      <c r="M229" t="n">
-        <v>5</v>
+      <c r="M229" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N229" t="n">
         <v>2</v>
@@ -16185,8 +16489,10 @@
       <c r="L233" t="n">
         <v>2</v>
       </c>
-      <c r="M233" t="n">
-        <v>4</v>
+      <c r="M233" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N233" t="n">
         <v>2</v>
@@ -16528,8 +16834,10 @@
       <c r="L238" t="n">
         <v>4</v>
       </c>
-      <c r="M238" t="n">
-        <v>4</v>
+      <c r="M238" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N238" t="n">
         <v>2</v>
@@ -16595,8 +16903,10 @@
       <c r="L239" t="n">
         <v>5</v>
       </c>
-      <c r="M239" t="n">
-        <v>4</v>
+      <c r="M239" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N239" t="n">
         <v>2</v>
@@ -16731,8 +17041,10 @@
       <c r="L241" t="n">
         <v>4</v>
       </c>
-      <c r="M241" t="n">
-        <v>4</v>
+      <c r="M241" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N241" t="n">
         <v>2</v>
@@ -16798,8 +17110,10 @@
       <c r="L242" t="n">
         <v>4</v>
       </c>
-      <c r="M242" t="n">
-        <v>4</v>
+      <c r="M242" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N242" t="n">
         <v>1</v>
@@ -16865,8 +17179,10 @@
       <c r="L243" t="n">
         <v>4</v>
       </c>
-      <c r="M243" t="n">
-        <v>3</v>
+      <c r="M243" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="N243" t="n">
         <v>0</v>
@@ -16932,8 +17248,10 @@
       <c r="L244" t="n">
         <v>4</v>
       </c>
-      <c r="M244" t="n">
-        <v>1</v>
+      <c r="M244" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N244" t="n">
         <v>1</v>
@@ -17068,8 +17386,10 @@
       <c r="L246" t="n">
         <v>4</v>
       </c>
-      <c r="M246" t="n">
-        <v>4</v>
+      <c r="M246" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N246" t="n">
         <v>2</v>
@@ -17135,8 +17455,10 @@
       <c r="L247" t="n">
         <v>3</v>
       </c>
-      <c r="M247" t="n">
-        <v>5</v>
+      <c r="M247" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N247" t="n">
         <v>2</v>
@@ -17202,8 +17524,10 @@
       <c r="L248" t="n">
         <v>2</v>
       </c>
-      <c r="M248" t="n">
-        <v>4</v>
+      <c r="M248" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N248" t="n">
         <v>2</v>
@@ -17407,8 +17731,10 @@
       <c r="L251" t="n">
         <v>4</v>
       </c>
-      <c r="M251" t="n">
-        <v>4</v>
+      <c r="M251" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N251" t="n">
         <v>2</v>
@@ -17474,8 +17800,10 @@
       <c r="L252" t="n">
         <v>4</v>
       </c>
-      <c r="M252" t="n">
-        <v>4</v>
+      <c r="M252" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N252" t="n">
         <v>2</v>
@@ -17541,8 +17869,10 @@
       <c r="L253" t="n">
         <v>4</v>
       </c>
-      <c r="M253" t="n">
-        <v>4</v>
+      <c r="M253" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N253" t="n">
         <v>1</v>
@@ -17815,8 +18145,10 @@
       <c r="L257" t="n">
         <v>4</v>
       </c>
-      <c r="M257" t="n">
-        <v>5</v>
+      <c r="M257" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N257" t="n">
         <v>1</v>
@@ -17882,8 +18214,10 @@
       <c r="L258" t="n">
         <v>4</v>
       </c>
-      <c r="M258" t="n">
-        <v>5</v>
+      <c r="M258" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N258" t="n">
         <v>2</v>
@@ -17949,8 +18283,10 @@
       <c r="L259" t="n">
         <v>5</v>
       </c>
-      <c r="M259" t="n">
-        <v>4</v>
+      <c r="M259" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N259" t="n">
         <v>0</v>
@@ -18016,8 +18352,10 @@
       <c r="L260" t="n">
         <v>2</v>
       </c>
-      <c r="M260" t="n">
-        <v>4</v>
+      <c r="M260" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N260" t="n">
         <v>2</v>
@@ -18083,8 +18421,10 @@
       <c r="L261" t="n">
         <v>5</v>
       </c>
-      <c r="M261" t="n">
-        <v>1</v>
+      <c r="M261" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N261" t="n">
         <v>2</v>
@@ -18150,8 +18490,10 @@
       <c r="L262" t="n">
         <v>4</v>
       </c>
-      <c r="M262" t="n">
-        <v>1</v>
+      <c r="M262" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N262" t="n">
         <v>2</v>
@@ -18217,8 +18559,10 @@
       <c r="L263" t="n">
         <v>5</v>
       </c>
-      <c r="M263" t="n">
-        <v>1</v>
+      <c r="M263" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N263" t="n">
         <v>2</v>
@@ -18284,8 +18628,10 @@
       <c r="L264" t="n">
         <v>4</v>
       </c>
-      <c r="M264" t="n">
-        <v>4</v>
+      <c r="M264" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N264" t="n">
         <v>2</v>
@@ -18420,8 +18766,10 @@
       <c r="L266" t="n">
         <v>5</v>
       </c>
-      <c r="M266" t="n">
-        <v>5</v>
+      <c r="M266" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N266" t="n">
         <v>2</v>
@@ -18487,8 +18835,10 @@
       <c r="L267" t="n">
         <v>3</v>
       </c>
-      <c r="M267" t="n">
-        <v>4</v>
+      <c r="M267" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N267" t="n">
         <v>2</v>
@@ -18554,8 +18904,10 @@
       <c r="L268" t="n">
         <v>4</v>
       </c>
-      <c r="M268" t="n">
-        <v>2</v>
+      <c r="M268" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="N268" t="n">
         <v>2</v>
@@ -18621,8 +18973,10 @@
       <c r="L269" t="n">
         <v>4</v>
       </c>
-      <c r="M269" t="n">
-        <v>5</v>
+      <c r="M269" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N269" t="n">
         <v>2</v>
@@ -18757,8 +19111,10 @@
       <c r="L271" t="n">
         <v>5</v>
       </c>
-      <c r="M271" t="n">
-        <v>4</v>
+      <c r="M271" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N271" t="n">
         <v>2</v>
@@ -18824,8 +19180,10 @@
       <c r="L272" t="n">
         <v>5</v>
       </c>
-      <c r="M272" t="n">
-        <v>5</v>
+      <c r="M272" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N272" t="n">
         <v>2</v>
@@ -18891,8 +19249,10 @@
       <c r="L273" t="n">
         <v>4</v>
       </c>
-      <c r="M273" t="n">
-        <v>4</v>
+      <c r="M273" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N273" t="n">
         <v>2</v>
@@ -19027,8 +19387,10 @@
       <c r="L275" t="n">
         <v>4</v>
       </c>
-      <c r="M275" t="n">
-        <v>4</v>
+      <c r="M275" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N275" t="n">
         <v>2</v>
@@ -19094,8 +19456,10 @@
       <c r="L276" t="n">
         <v>4</v>
       </c>
-      <c r="M276" t="n">
-        <v>4</v>
+      <c r="M276" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N276" t="n">
         <v>2</v>
@@ -19161,8 +19525,10 @@
       <c r="L277" t="n">
         <v>5</v>
       </c>
-      <c r="M277" t="n">
-        <v>1</v>
+      <c r="M277" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N277" t="n">
         <v>2</v>
@@ -19228,8 +19594,10 @@
       <c r="L278" t="n">
         <v>4</v>
       </c>
-      <c r="M278" t="n">
-        <v>4</v>
+      <c r="M278" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N278" t="n">
         <v>2</v>
@@ -19295,8 +19663,10 @@
       <c r="L279" t="n">
         <v>4</v>
       </c>
-      <c r="M279" t="n">
-        <v>1</v>
+      <c r="M279" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N279" t="n">
         <v>1</v>
@@ -19362,8 +19732,10 @@
       <c r="L280" t="n">
         <v>4</v>
       </c>
-      <c r="M280" t="n">
-        <v>4</v>
+      <c r="M280" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N280" t="n">
         <v>2</v>
@@ -19429,8 +19801,10 @@
       <c r="L281" t="n">
         <v>4</v>
       </c>
-      <c r="M281" t="n">
-        <v>2</v>
+      <c r="M281" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="N281" t="n">
         <v>2</v>
@@ -19496,8 +19870,10 @@
       <c r="L282" t="n">
         <v>5</v>
       </c>
-      <c r="M282" t="n">
-        <v>1</v>
+      <c r="M282" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N282" t="n">
         <v>2</v>
@@ -19563,8 +19939,10 @@
       <c r="L283" t="n">
         <v>4</v>
       </c>
-      <c r="M283" t="n">
-        <v>4</v>
+      <c r="M283" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N283" t="n">
         <v>2</v>
@@ -19630,8 +20008,10 @@
       <c r="L284" t="n">
         <v>4</v>
       </c>
-      <c r="M284" t="n">
-        <v>4</v>
+      <c r="M284" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N284" t="n">
         <v>1</v>
@@ -19697,8 +20077,10 @@
       <c r="L285" t="n">
         <v>2</v>
       </c>
-      <c r="M285" t="n">
-        <v>4</v>
+      <c r="M285" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N285" t="n">
         <v>2</v>
@@ -19764,8 +20146,10 @@
       <c r="L286" t="n">
         <v>3</v>
       </c>
-      <c r="M286" t="n">
-        <v>5</v>
+      <c r="M286" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N286" t="n">
         <v>2</v>
@@ -19831,8 +20215,10 @@
       <c r="L287" t="n">
         <v>2</v>
       </c>
-      <c r="M287" t="n">
-        <v>4</v>
+      <c r="M287" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N287" t="n">
         <v>2</v>
@@ -19898,8 +20284,10 @@
       <c r="L288" t="n">
         <v>3</v>
       </c>
-      <c r="M288" t="n">
-        <v>4</v>
+      <c r="M288" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N288" t="n">
         <v>2</v>
@@ -20103,8 +20491,10 @@
       <c r="L291" t="n">
         <v>3</v>
       </c>
-      <c r="M291" t="n">
-        <v>4</v>
+      <c r="M291" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N291" t="n">
         <v>2</v>
@@ -20170,8 +20560,10 @@
       <c r="L292" t="n">
         <v>2</v>
       </c>
-      <c r="M292" t="n">
-        <v>4</v>
+      <c r="M292" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N292" t="n">
         <v>2</v>
@@ -20237,8 +20629,10 @@
       <c r="L293" t="n">
         <v>3</v>
       </c>
-      <c r="M293" t="n">
-        <v>4</v>
+      <c r="M293" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N293" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
resolve set loc data type
</commit_message>
<xml_diff>
--- a/data/split/test.xlsx
+++ b/data/split/test.xlsx
@@ -570,8 +570,10 @@
       <c r="L2" t="n">
         <v>4</v>
       </c>
-      <c r="M2" t="n">
-        <v>4</v>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N2" t="n">
         <v>2</v>
@@ -649,8 +651,10 @@
       <c r="L3" t="n">
         <v>5</v>
       </c>
-      <c r="M3" t="n">
-        <v>1</v>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N3" t="n">
         <v>2</v>
@@ -728,8 +732,10 @@
       <c r="L4" t="n">
         <v>5</v>
       </c>
-      <c r="M4" t="n">
-        <v>4</v>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N4" t="n">
         <v>1</v>
@@ -807,8 +813,10 @@
       <c r="L5" t="n">
         <v>5</v>
       </c>
-      <c r="M5" t="n">
-        <v>4</v>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N5" t="n">
         <v>1</v>
@@ -886,8 +894,10 @@
       <c r="L6" t="n">
         <v>3</v>
       </c>
-      <c r="M6" t="n">
-        <v>4</v>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N6" t="n">
         <v>2</v>
@@ -965,8 +975,10 @@
       <c r="L7" t="n">
         <v>2</v>
       </c>
-      <c r="M7" t="n">
-        <v>5</v>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N7" t="n">
         <v>2</v>
@@ -1044,8 +1056,10 @@
       <c r="L8" t="n">
         <v>5</v>
       </c>
-      <c r="M8" t="n">
-        <v>1</v>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N8" t="n">
         <v>2</v>
@@ -1123,8 +1137,10 @@
       <c r="L9" t="n">
         <v>2</v>
       </c>
-      <c r="M9" t="n">
-        <v>3</v>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="N9" t="n">
         <v>2</v>
@@ -1202,8 +1218,10 @@
       <c r="L10" t="n">
         <v>4</v>
       </c>
-      <c r="M10" t="n">
-        <v>4</v>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N10" t="n">
         <v>2</v>
@@ -1281,8 +1299,10 @@
       <c r="L11" t="n">
         <v>4</v>
       </c>
-      <c r="M11" t="n">
-        <v>1</v>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N11" t="n">
         <v>1</v>
@@ -1522,8 +1542,10 @@
       <c r="L14" t="n">
         <v>4</v>
       </c>
-      <c r="M14" t="n">
-        <v>4</v>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N14" t="n">
         <v>2</v>
@@ -1763,8 +1785,10 @@
       <c r="L17" t="n">
         <v>3</v>
       </c>
-      <c r="M17" t="n">
-        <v>4</v>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N17" t="n">
         <v>1</v>
@@ -2004,8 +2028,10 @@
       <c r="L20" t="n">
         <v>4</v>
       </c>
-      <c r="M20" t="n">
-        <v>1</v>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N20" t="n">
         <v>1</v>
@@ -2083,8 +2109,10 @@
       <c r="L21" t="n">
         <v>2</v>
       </c>
-      <c r="M21" t="n">
-        <v>4</v>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N21" t="n">
         <v>3</v>
@@ -2243,8 +2271,10 @@
       <c r="L23" t="n">
         <v>4</v>
       </c>
-      <c r="M23" t="n">
-        <v>4</v>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N23" t="n">
         <v>2</v>
@@ -2322,8 +2352,10 @@
       <c r="L24" t="n">
         <v>5</v>
       </c>
-      <c r="M24" t="n">
-        <v>4</v>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N24" t="n">
         <v>2</v>
@@ -2482,8 +2514,10 @@
       <c r="L26" t="n">
         <v>4</v>
       </c>
-      <c r="M26" t="n">
-        <v>4</v>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N26" t="n">
         <v>2</v>
@@ -2723,8 +2757,10 @@
       <c r="L29" t="n">
         <v>4</v>
       </c>
-      <c r="M29" t="n">
-        <v>4</v>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N29" t="n">
         <v>2</v>
@@ -2802,8 +2838,10 @@
       <c r="L30" t="n">
         <v>4</v>
       </c>
-      <c r="M30" t="n">
-        <v>4</v>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N30" t="n">
         <v>2</v>
@@ -2881,8 +2919,10 @@
       <c r="L31" t="n">
         <v>4</v>
       </c>
-      <c r="M31" t="n">
-        <v>4</v>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N31" t="n">
         <v>2</v>
@@ -3122,8 +3162,10 @@
       <c r="L34" t="n">
         <v>5</v>
       </c>
-      <c r="M34" t="n">
-        <v>4</v>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N34" t="n">
         <v>1</v>
@@ -3201,8 +3243,10 @@
       <c r="L35" t="n">
         <v>4</v>
       </c>
-      <c r="M35" t="n">
-        <v>5</v>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N35" t="n">
         <v>2</v>
@@ -3280,8 +3324,10 @@
       <c r="L36" t="n">
         <v>3</v>
       </c>
-      <c r="M36" t="n">
-        <v>4</v>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N36" t="n">
         <v>2</v>
@@ -3440,8 +3486,10 @@
       <c r="L38" t="n">
         <v>4</v>
       </c>
-      <c r="M38" t="n">
-        <v>3</v>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="N38" t="n">
         <v>2</v>
@@ -3681,8 +3729,10 @@
       <c r="L41" t="n">
         <v>5</v>
       </c>
-      <c r="M41" t="n">
-        <v>1</v>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N41" t="n">
         <v>0</v>
@@ -3841,8 +3891,10 @@
       <c r="L43" t="n">
         <v>4</v>
       </c>
-      <c r="M43" t="n">
-        <v>4</v>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N43" t="n">
         <v>2</v>
@@ -3920,8 +3972,10 @@
       <c r="L44" t="n">
         <v>4</v>
       </c>
-      <c r="M44" t="n">
-        <v>4</v>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N44" t="n">
         <v>2</v>
@@ -3999,8 +4053,10 @@
       <c r="L45" t="n">
         <v>4</v>
       </c>
-      <c r="M45" t="n">
-        <v>4</v>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N45" t="n">
         <v>2</v>
@@ -4078,8 +4134,10 @@
       <c r="L46" t="n">
         <v>5</v>
       </c>
-      <c r="M46" t="n">
-        <v>4</v>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N46" t="n">
         <v>2</v>
@@ -4157,8 +4215,10 @@
       <c r="L47" t="n">
         <v>3</v>
       </c>
-      <c r="M47" t="n">
-        <v>4</v>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N47" t="n">
         <v>2</v>
@@ -4236,8 +4296,10 @@
       <c r="L48" t="n">
         <v>4</v>
       </c>
-      <c r="M48" t="n">
-        <v>4</v>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N48" t="n">
         <v>2</v>
@@ -4477,8 +4539,10 @@
       <c r="L51" t="n">
         <v>5</v>
       </c>
-      <c r="M51" t="n">
-        <v>1</v>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N51" t="n">
         <v>2</v>
@@ -4556,8 +4620,10 @@
       <c r="L52" t="n">
         <v>4</v>
       </c>
-      <c r="M52" t="n">
-        <v>4</v>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N52" t="n">
         <v>2</v>
@@ -4716,8 +4782,10 @@
       <c r="L54" t="n">
         <v>5</v>
       </c>
-      <c r="M54" t="n">
-        <v>2</v>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="N54" t="n">
         <v>2</v>
@@ -4876,8 +4944,10 @@
       <c r="L56" t="n">
         <v>4</v>
       </c>
-      <c r="M56" t="n">
-        <v>4</v>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N56" t="n">
         <v>2</v>
@@ -4955,8 +5025,10 @@
       <c r="L57" t="n">
         <v>4</v>
       </c>
-      <c r="M57" t="n">
-        <v>1</v>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N57" t="n">
         <v>1</v>
@@ -5034,8 +5106,10 @@
       <c r="L58" t="n">
         <v>5</v>
       </c>
-      <c r="M58" t="n">
-        <v>1</v>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N58" t="n">
         <v>1</v>
@@ -5113,8 +5187,10 @@
       <c r="L59" t="n">
         <v>3</v>
       </c>
-      <c r="M59" t="n">
-        <v>5</v>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N59" t="n">
         <v>1</v>
@@ -5273,8 +5349,10 @@
       <c r="L61" t="n">
         <v>5</v>
       </c>
-      <c r="M61" t="n">
-        <v>1</v>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N61" t="n">
         <v>1</v>
@@ -5433,8 +5511,10 @@
       <c r="L63" t="n">
         <v>4</v>
       </c>
-      <c r="M63" t="n">
-        <v>5</v>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N63" t="n">
         <v>2</v>
@@ -5512,8 +5592,10 @@
       <c r="L64" t="n">
         <v>2</v>
       </c>
-      <c r="M64" t="n">
-        <v>5</v>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N64" t="n">
         <v>2</v>
@@ -5591,8 +5673,10 @@
       <c r="L65" t="n">
         <v>4</v>
       </c>
-      <c r="M65" t="n">
-        <v>5</v>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N65" t="n">
         <v>2</v>
@@ -5751,8 +5835,10 @@
       <c r="L67" t="n">
         <v>4</v>
       </c>
-      <c r="M67" t="n">
-        <v>5</v>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N67" t="n">
         <v>2</v>
@@ -5830,8 +5916,10 @@
       <c r="L68" t="n">
         <v>2</v>
       </c>
-      <c r="M68" t="n">
-        <v>4</v>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N68" t="n">
         <v>3</v>
@@ -5909,8 +5997,10 @@
       <c r="L69" t="n">
         <v>2</v>
       </c>
-      <c r="M69" t="n">
-        <v>5</v>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N69" t="n">
         <v>3</v>
@@ -5988,8 +6078,10 @@
       <c r="L70" t="n">
         <v>4</v>
       </c>
-      <c r="M70" t="n">
-        <v>4</v>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N70" t="n">
         <v>2</v>
@@ -6067,8 +6159,10 @@
       <c r="L71" t="n">
         <v>4</v>
       </c>
-      <c r="M71" t="n">
-        <v>4</v>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N71" t="n">
         <v>2</v>
@@ -6146,8 +6240,10 @@
       <c r="L72" t="n">
         <v>5</v>
       </c>
-      <c r="M72" t="n">
-        <v>1</v>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N72" t="n">
         <v>2</v>
@@ -6306,8 +6402,10 @@
       <c r="L74" t="n">
         <v>2</v>
       </c>
-      <c r="M74" t="n">
-        <v>3</v>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="N74" t="n">
         <v>2</v>
@@ -6385,8 +6483,10 @@
       <c r="L75" t="n">
         <v>4</v>
       </c>
-      <c r="M75" t="n">
-        <v>2</v>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="N75" t="n">
         <v>1</v>
@@ -6626,8 +6726,10 @@
       <c r="L78" t="n">
         <v>2</v>
       </c>
-      <c r="M78" t="n">
-        <v>4</v>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N78" t="n">
         <v>2</v>
@@ -6705,8 +6807,10 @@
       <c r="L79" t="n">
         <v>4</v>
       </c>
-      <c r="M79" t="n">
-        <v>4</v>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N79" t="n">
         <v>2</v>
@@ -6784,8 +6888,10 @@
       <c r="L80" t="n">
         <v>4</v>
       </c>
-      <c r="M80" t="n">
-        <v>5</v>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N80" t="n">
         <v>2</v>
@@ -6863,8 +6969,10 @@
       <c r="L81" t="n">
         <v>2</v>
       </c>
-      <c r="M81" t="n">
-        <v>4</v>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N81" t="n">
         <v>2</v>
@@ -6942,8 +7050,10 @@
       <c r="L82" t="n">
         <v>5</v>
       </c>
-      <c r="M82" t="n">
-        <v>4</v>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N82" t="n">
         <v>2</v>
@@ -7021,8 +7131,10 @@
       <c r="L83" t="n">
         <v>4</v>
       </c>
-      <c r="M83" t="n">
-        <v>1</v>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N83" t="n">
         <v>1</v>
@@ -7100,8 +7212,10 @@
       <c r="L84" t="n">
         <v>4</v>
       </c>
-      <c r="M84" t="n">
-        <v>4</v>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N84" t="n">
         <v>1</v>
@@ -7260,8 +7374,10 @@
       <c r="L86" t="n">
         <v>2</v>
       </c>
-      <c r="M86" t="n">
-        <v>4</v>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N86" t="n">
         <v>2</v>
@@ -7339,8 +7455,10 @@
       <c r="L87" t="n">
         <v>2</v>
       </c>
-      <c r="M87" t="n">
-        <v>4</v>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N87" t="n">
         <v>3</v>
@@ -7418,8 +7536,10 @@
       <c r="L88" t="n">
         <v>4</v>
       </c>
-      <c r="M88" t="n">
-        <v>4</v>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N88" t="n">
         <v>2</v>
@@ -7578,8 +7698,10 @@
       <c r="L90" t="n">
         <v>4</v>
       </c>
-      <c r="M90" t="n">
-        <v>4</v>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N90" t="n">
         <v>2</v>
@@ -7657,8 +7779,10 @@
       <c r="L91" t="n">
         <v>3</v>
       </c>
-      <c r="M91" t="n">
-        <v>4</v>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N91" t="n">
         <v>2</v>
@@ -7898,8 +8022,10 @@
       <c r="L94" t="n">
         <v>4</v>
       </c>
-      <c r="M94" t="n">
-        <v>4</v>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N94" t="n">
         <v>2</v>
@@ -7977,8 +8103,10 @@
       <c r="L95" t="n">
         <v>5</v>
       </c>
-      <c r="M95" t="n">
-        <v>4</v>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N95" t="n">
         <v>2</v>
@@ -8056,8 +8184,10 @@
       <c r="L96" t="n">
         <v>3</v>
       </c>
-      <c r="M96" t="n">
-        <v>5</v>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N96" t="n">
         <v>2</v>
@@ -8216,8 +8346,10 @@
       <c r="L98" t="n">
         <v>4</v>
       </c>
-      <c r="M98" t="n">
-        <v>4</v>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N98" t="n">
         <v>2</v>
@@ -8295,8 +8427,10 @@
       <c r="L99" t="n">
         <v>5</v>
       </c>
-      <c r="M99" t="n">
-        <v>5</v>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N99" t="n">
         <v>2</v>
@@ -8374,8 +8508,10 @@
       <c r="L100" t="n">
         <v>4</v>
       </c>
-      <c r="M100" t="n">
-        <v>5</v>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N100" t="n">
         <v>2</v>
@@ -8453,8 +8589,10 @@
       <c r="L101" t="n">
         <v>5</v>
       </c>
-      <c r="M101" t="n">
-        <v>3</v>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="N101" t="n">
         <v>2</v>
@@ -8694,8 +8832,10 @@
       <c r="L104" t="n">
         <v>5</v>
       </c>
-      <c r="M104" t="n">
-        <v>5</v>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N104" t="n">
         <v>2</v>
@@ -8773,8 +8913,10 @@
       <c r="L105" t="n">
         <v>4</v>
       </c>
-      <c r="M105" t="n">
-        <v>4</v>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N105" t="n">
         <v>2</v>
@@ -8852,8 +8994,10 @@
       <c r="L106" t="n">
         <v>4</v>
       </c>
-      <c r="M106" t="n">
-        <v>4</v>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N106" t="n">
         <v>2</v>
@@ -8931,8 +9075,10 @@
       <c r="L107" t="n">
         <v>4</v>
       </c>
-      <c r="M107" t="n">
-        <v>4</v>
+      <c r="M107" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N107" t="n">
         <v>2</v>
@@ -9010,8 +9156,10 @@
       <c r="L108" t="n">
         <v>4</v>
       </c>
-      <c r="M108" t="n">
-        <v>4</v>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N108" t="n">
         <v>2</v>
@@ -9089,8 +9237,10 @@
       <c r="L109" t="n">
         <v>2</v>
       </c>
-      <c r="M109" t="n">
-        <v>4</v>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N109" t="n">
         <v>2</v>
@@ -9249,8 +9399,10 @@
       <c r="L111" t="n">
         <v>5</v>
       </c>
-      <c r="M111" t="n">
-        <v>4</v>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N111" t="n">
         <v>2</v>
@@ -9409,8 +9561,10 @@
       <c r="L113" t="n">
         <v>4</v>
       </c>
-      <c r="M113" t="n">
-        <v>4</v>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N113" t="n">
         <v>2</v>
@@ -9488,8 +9642,10 @@
       <c r="L114" t="n">
         <v>3</v>
       </c>
-      <c r="M114" t="n">
-        <v>4</v>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N114" t="n">
         <v>2</v>
@@ -9567,8 +9723,10 @@
       <c r="L115" t="n">
         <v>2</v>
       </c>
-      <c r="M115" t="n">
-        <v>5</v>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N115" t="n">
         <v>2</v>
@@ -9646,8 +9804,10 @@
       <c r="L116" t="n">
         <v>1</v>
       </c>
-      <c r="M116" t="n">
-        <v>5</v>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N116" t="n">
         <v>2</v>
@@ -9806,8 +9966,10 @@
       <c r="L118" t="n">
         <v>5</v>
       </c>
-      <c r="M118" t="n">
-        <v>4</v>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N118" t="n">
         <v>2</v>
@@ -9885,8 +10047,10 @@
       <c r="L119" t="n">
         <v>2</v>
       </c>
-      <c r="M119" t="n">
-        <v>4</v>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N119" t="n">
         <v>2</v>
@@ -10045,8 +10209,10 @@
       <c r="L121" t="n">
         <v>5</v>
       </c>
-      <c r="M121" t="n">
-        <v>4</v>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N121" t="n">
         <v>2</v>
@@ -10124,8 +10290,10 @@
       <c r="L122" t="n">
         <v>4</v>
       </c>
-      <c r="M122" t="n">
-        <v>5</v>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N122" t="n">
         <v>1</v>
@@ -10203,8 +10371,10 @@
       <c r="L123" t="n">
         <v>3</v>
       </c>
-      <c r="M123" t="n">
-        <v>4</v>
+      <c r="M123" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N123" t="n">
         <v>2</v>
@@ -10444,8 +10614,10 @@
       <c r="L126" t="n">
         <v>5</v>
       </c>
-      <c r="M126" t="n">
-        <v>4</v>
+      <c r="M126" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N126" t="n">
         <v>2</v>
@@ -10523,8 +10695,10 @@
       <c r="L127" t="n">
         <v>3</v>
       </c>
-      <c r="M127" t="n">
-        <v>1</v>
+      <c r="M127" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N127" t="n">
         <v>0</v>
@@ -10683,8 +10857,10 @@
       <c r="L129" t="n">
         <v>2</v>
       </c>
-      <c r="M129" t="n">
-        <v>4</v>
+      <c r="M129" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N129" t="n">
         <v>2</v>
@@ -10762,8 +10938,10 @@
       <c r="L130" t="n">
         <v>5</v>
       </c>
-      <c r="M130" t="n">
-        <v>4</v>
+      <c r="M130" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N130" t="n">
         <v>2</v>
@@ -10922,8 +11100,10 @@
       <c r="L132" t="n">
         <v>4</v>
       </c>
-      <c r="M132" t="n">
-        <v>4</v>
+      <c r="M132" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N132" t="n">
         <v>2</v>
@@ -11001,8 +11181,10 @@
       <c r="L133" t="n">
         <v>5</v>
       </c>
-      <c r="M133" t="n">
-        <v>1</v>
+      <c r="M133" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N133" t="n">
         <v>2</v>
@@ -11242,8 +11424,10 @@
       <c r="L136" t="n">
         <v>3</v>
       </c>
-      <c r="M136" t="n">
-        <v>1</v>
+      <c r="M136" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N136" t="n">
         <v>2</v>
@@ -11321,8 +11505,10 @@
       <c r="L137" t="n">
         <v>4</v>
       </c>
-      <c r="M137" t="n">
-        <v>4</v>
+      <c r="M137" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N137" t="n">
         <v>2</v>
@@ -11400,8 +11586,10 @@
       <c r="L138" t="n">
         <v>4</v>
       </c>
-      <c r="M138" t="n">
-        <v>3</v>
+      <c r="M138" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="N138" t="n">
         <v>2</v>
@@ -11479,8 +11667,10 @@
       <c r="L139" t="n">
         <v>2</v>
       </c>
-      <c r="M139" t="n">
-        <v>4</v>
+      <c r="M139" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N139" t="n">
         <v>2</v>
@@ -11639,8 +11829,10 @@
       <c r="L141" t="n">
         <v>5</v>
       </c>
-      <c r="M141" t="n">
-        <v>4</v>
+      <c r="M141" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N141" t="n">
         <v>1</v>
@@ -11718,8 +11910,10 @@
       <c r="L142" t="n">
         <v>5</v>
       </c>
-      <c r="M142" t="n">
-        <v>4</v>
+      <c r="M142" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N142" t="n">
         <v>2</v>
@@ -11797,8 +11991,10 @@
       <c r="L143" t="n">
         <v>4</v>
       </c>
-      <c r="M143" t="n">
-        <v>1</v>
+      <c r="M143" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N143" t="n">
         <v>0</v>
@@ -12119,8 +12315,10 @@
       <c r="L147" t="n">
         <v>5</v>
       </c>
-      <c r="M147" t="n">
-        <v>4</v>
+      <c r="M147" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N147" t="n">
         <v>1</v>
@@ -12198,8 +12396,10 @@
       <c r="L148" t="n">
         <v>4</v>
       </c>
-      <c r="M148" t="n">
-        <v>1</v>
+      <c r="M148" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N148" t="n">
         <v>2</v>
@@ -12358,8 +12558,10 @@
       <c r="L150" t="n">
         <v>3</v>
       </c>
-      <c r="M150" t="n">
-        <v>3</v>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="N150" t="n">
         <v>2</v>
@@ -12437,8 +12639,10 @@
       <c r="L151" t="n">
         <v>5</v>
       </c>
-      <c r="M151" t="n">
-        <v>4</v>
+      <c r="M151" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N151" t="n">
         <v>1</v>
@@ -12678,8 +12882,10 @@
       <c r="L154" t="n">
         <v>4</v>
       </c>
-      <c r="M154" t="n">
-        <v>4</v>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N154" t="n">
         <v>2</v>
@@ -12757,8 +12963,10 @@
       <c r="L155" t="n">
         <v>4</v>
       </c>
-      <c r="M155" t="n">
-        <v>2</v>
+      <c r="M155" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="N155" t="n">
         <v>2</v>
@@ -12917,8 +13125,10 @@
       <c r="L157" t="n">
         <v>5</v>
       </c>
-      <c r="M157" t="n">
-        <v>4</v>
+      <c r="M157" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N157" t="n">
         <v>2</v>
@@ -12996,8 +13206,10 @@
       <c r="L158" t="n">
         <v>4</v>
       </c>
-      <c r="M158" t="n">
-        <v>5</v>
+      <c r="M158" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N158" t="n">
         <v>2</v>
@@ -13075,8 +13287,10 @@
       <c r="L159" t="n">
         <v>3</v>
       </c>
-      <c r="M159" t="n">
-        <v>4</v>
+      <c r="M159" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N159" t="n">
         <v>2</v>
@@ -13316,8 +13530,10 @@
       <c r="L162" t="n">
         <v>5</v>
       </c>
-      <c r="M162" t="n">
-        <v>1</v>
+      <c r="M162" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N162" t="n">
         <v>1</v>
@@ -13395,8 +13611,10 @@
       <c r="L163" t="n">
         <v>4</v>
       </c>
-      <c r="M163" t="n">
-        <v>4</v>
+      <c r="M163" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N163" t="n">
         <v>2</v>
@@ -13474,8 +13692,10 @@
       <c r="L164" t="n">
         <v>4</v>
       </c>
-      <c r="M164" t="n">
-        <v>4</v>
+      <c r="M164" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N164" t="n">
         <v>2</v>
@@ -13553,8 +13773,10 @@
       <c r="L165" t="n">
         <v>2</v>
       </c>
-      <c r="M165" t="n">
-        <v>4</v>
+      <c r="M165" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N165" t="n">
         <v>2</v>
@@ -13632,8 +13854,10 @@
       <c r="L166" t="n">
         <v>5</v>
       </c>
-      <c r="M166" t="n">
-        <v>4</v>
+      <c r="M166" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N166" t="n">
         <v>1</v>
@@ -13711,8 +13935,10 @@
       <c r="L167" t="n">
         <v>2</v>
       </c>
-      <c r="M167" t="n">
-        <v>4</v>
+      <c r="M167" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N167" t="n">
         <v>0</v>
@@ -13790,8 +14016,10 @@
       <c r="L168" t="n">
         <v>5</v>
       </c>
-      <c r="M168" t="n">
-        <v>1</v>
+      <c r="M168" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N168" t="n">
         <v>2</v>
@@ -13950,8 +14178,10 @@
       <c r="L170" t="n">
         <v>4</v>
       </c>
-      <c r="M170" t="n">
-        <v>4</v>
+      <c r="M170" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N170" t="n">
         <v>2</v>
@@ -14029,8 +14259,10 @@
       <c r="L171" t="n">
         <v>4</v>
       </c>
-      <c r="M171" t="n">
-        <v>4</v>
+      <c r="M171" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N171" t="n">
         <v>2</v>
@@ -14108,8 +14340,10 @@
       <c r="L172" t="n">
         <v>4</v>
       </c>
-      <c r="M172" t="n">
-        <v>4</v>
+      <c r="M172" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N172" t="n">
         <v>0</v>
@@ -14268,8 +14502,10 @@
       <c r="L174" t="n">
         <v>4</v>
       </c>
-      <c r="M174" t="n">
-        <v>4</v>
+      <c r="M174" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N174" t="n">
         <v>2</v>
@@ -14590,8 +14826,10 @@
       <c r="L178" t="n">
         <v>2</v>
       </c>
-      <c r="M178" t="n">
-        <v>5</v>
+      <c r="M178" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N178" t="n">
         <v>2</v>
@@ -14669,8 +14907,10 @@
       <c r="L179" t="n">
         <v>4</v>
       </c>
-      <c r="M179" t="n">
-        <v>4</v>
+      <c r="M179" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N179" t="n">
         <v>2</v>
@@ -14829,8 +15069,10 @@
       <c r="L181" t="n">
         <v>4</v>
       </c>
-      <c r="M181" t="n">
-        <v>5</v>
+      <c r="M181" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N181" t="n">
         <v>2</v>
@@ -14908,8 +15150,10 @@
       <c r="L182" t="n">
         <v>5</v>
       </c>
-      <c r="M182" t="n">
-        <v>5</v>
+      <c r="M182" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N182" t="n">
         <v>2</v>
@@ -14987,8 +15231,10 @@
       <c r="L183" t="n">
         <v>3</v>
       </c>
-      <c r="M183" t="n">
-        <v>4</v>
+      <c r="M183" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N183" t="n">
         <v>2</v>
@@ -15066,8 +15312,10 @@
       <c r="L184" t="n">
         <v>4</v>
       </c>
-      <c r="M184" t="n">
-        <v>5</v>
+      <c r="M184" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N184" t="n">
         <v>1</v>
@@ -15388,8 +15636,10 @@
       <c r="L188" t="n">
         <v>2</v>
       </c>
-      <c r="M188" t="n">
-        <v>4</v>
+      <c r="M188" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N188" t="n">
         <v>3</v>
@@ -15548,8 +15798,10 @@
       <c r="L190" t="n">
         <v>2</v>
       </c>
-      <c r="M190" t="n">
-        <v>4</v>
+      <c r="M190" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N190" t="n">
         <v>3</v>
@@ -15627,8 +15879,10 @@
       <c r="L191" t="n">
         <v>3</v>
       </c>
-      <c r="M191" t="n">
-        <v>4</v>
+      <c r="M191" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N191" t="n">
         <v>2</v>
@@ -15706,8 +15960,10 @@
       <c r="L192" t="n">
         <v>5</v>
       </c>
-      <c r="M192" t="n">
-        <v>1</v>
+      <c r="M192" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N192" t="n">
         <v>2</v>
@@ -15785,8 +16041,10 @@
       <c r="L193" t="n">
         <v>4</v>
       </c>
-      <c r="M193" t="n">
-        <v>4</v>
+      <c r="M193" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N193" t="n">
         <v>2</v>
@@ -15945,8 +16203,10 @@
       <c r="L195" t="n">
         <v>3</v>
       </c>
-      <c r="M195" t="n">
-        <v>4</v>
+      <c r="M195" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N195" t="n">
         <v>2</v>
@@ -16024,8 +16284,10 @@
       <c r="L196" t="n">
         <v>5</v>
       </c>
-      <c r="M196" t="n">
-        <v>4</v>
+      <c r="M196" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N196" t="n">
         <v>2</v>
@@ -16184,8 +16446,10 @@
       <c r="L198" t="n">
         <v>2</v>
       </c>
-      <c r="M198" t="n">
-        <v>4</v>
+      <c r="M198" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N198" t="n">
         <v>2</v>
@@ -16344,8 +16608,10 @@
       <c r="L200" t="n">
         <v>4</v>
       </c>
-      <c r="M200" t="n">
-        <v>4</v>
+      <c r="M200" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N200" t="n">
         <v>2</v>
@@ -16423,8 +16689,10 @@
       <c r="L201" t="n">
         <v>4</v>
       </c>
-      <c r="M201" t="n">
-        <v>4</v>
+      <c r="M201" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N201" t="n">
         <v>2</v>
@@ -16502,8 +16770,10 @@
       <c r="L202" t="n">
         <v>2</v>
       </c>
-      <c r="M202" t="n">
-        <v>4</v>
+      <c r="M202" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N202" t="n">
         <v>1</v>
@@ -16581,8 +16851,10 @@
       <c r="L203" t="n">
         <v>5</v>
       </c>
-      <c r="M203" t="n">
-        <v>1</v>
+      <c r="M203" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N203" t="n">
         <v>1</v>
@@ -16741,8 +17013,10 @@
       <c r="L205" t="n">
         <v>3</v>
       </c>
-      <c r="M205" t="n">
-        <v>4</v>
+      <c r="M205" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N205" t="n">
         <v>2</v>
@@ -16901,8 +17175,10 @@
       <c r="L207" t="n">
         <v>4</v>
       </c>
-      <c r="M207" t="n">
-        <v>4</v>
+      <c r="M207" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N207" t="n">
         <v>2</v>
@@ -17061,8 +17337,10 @@
       <c r="L209" t="n">
         <v>2</v>
       </c>
-      <c r="M209" t="n">
-        <v>4</v>
+      <c r="M209" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N209" t="n">
         <v>3</v>
@@ -17221,8 +17499,10 @@
       <c r="L211" t="n">
         <v>4</v>
       </c>
-      <c r="M211" t="n">
-        <v>4</v>
+      <c r="M211" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N211" t="n">
         <v>2</v>
@@ -17300,8 +17580,10 @@
       <c r="L212" t="n">
         <v>2</v>
       </c>
-      <c r="M212" t="n">
-        <v>4</v>
+      <c r="M212" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N212" t="n">
         <v>2</v>
@@ -17379,8 +17661,10 @@
       <c r="L213" t="n">
         <v>4</v>
       </c>
-      <c r="M213" t="n">
-        <v>4</v>
+      <c r="M213" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N213" t="n">
         <v>2</v>
@@ -17458,8 +17742,10 @@
       <c r="L214" t="n">
         <v>4</v>
       </c>
-      <c r="M214" t="n">
-        <v>5</v>
+      <c r="M214" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N214" t="n">
         <v>2</v>
@@ -17699,8 +17985,10 @@
       <c r="L217" t="n">
         <v>5</v>
       </c>
-      <c r="M217" t="n">
-        <v>4</v>
+      <c r="M217" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N217" t="n">
         <v>2</v>
@@ -17859,8 +18147,10 @@
       <c r="L219" t="n">
         <v>5</v>
       </c>
-      <c r="M219" t="n">
-        <v>5</v>
+      <c r="M219" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N219" t="n">
         <v>2</v>
@@ -17938,8 +18228,10 @@
       <c r="L220" t="n">
         <v>5</v>
       </c>
-      <c r="M220" t="n">
-        <v>4</v>
+      <c r="M220" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N220" t="n">
         <v>2</v>
@@ -18098,8 +18390,10 @@
       <c r="L222" t="n">
         <v>2</v>
       </c>
-      <c r="M222" t="n">
-        <v>4</v>
+      <c r="M222" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N222" t="n">
         <v>3</v>
@@ -18258,8 +18552,10 @@
       <c r="L224" t="n">
         <v>3</v>
       </c>
-      <c r="M224" t="n">
-        <v>5</v>
+      <c r="M224" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N224" t="n">
         <v>2</v>
@@ -18337,8 +18633,10 @@
       <c r="L225" t="n">
         <v>4</v>
       </c>
-      <c r="M225" t="n">
-        <v>4</v>
+      <c r="M225" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N225" t="n">
         <v>2</v>
@@ -18497,8 +18795,10 @@
       <c r="L227" t="n">
         <v>4</v>
       </c>
-      <c r="M227" t="n">
-        <v>4</v>
+      <c r="M227" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N227" t="n">
         <v>2</v>
@@ -18576,8 +18876,10 @@
       <c r="L228" t="n">
         <v>4</v>
       </c>
-      <c r="M228" t="n">
-        <v>4</v>
+      <c r="M228" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N228" t="n">
         <v>2</v>
@@ -18655,8 +18957,10 @@
       <c r="L229" t="n">
         <v>3</v>
       </c>
-      <c r="M229" t="n">
-        <v>5</v>
+      <c r="M229" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N229" t="n">
         <v>2</v>
@@ -18977,8 +19281,10 @@
       <c r="L233" t="n">
         <v>2</v>
       </c>
-      <c r="M233" t="n">
-        <v>4</v>
+      <c r="M233" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N233" t="n">
         <v>2</v>
@@ -19380,8 +19686,10 @@
       <c r="L238" t="n">
         <v>4</v>
       </c>
-      <c r="M238" t="n">
-        <v>4</v>
+      <c r="M238" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N238" t="n">
         <v>2</v>
@@ -19459,8 +19767,10 @@
       <c r="L239" t="n">
         <v>5</v>
       </c>
-      <c r="M239" t="n">
-        <v>4</v>
+      <c r="M239" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N239" t="n">
         <v>2</v>
@@ -19619,8 +19929,10 @@
       <c r="L241" t="n">
         <v>4</v>
       </c>
-      <c r="M241" t="n">
-        <v>4</v>
+      <c r="M241" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N241" t="n">
         <v>2</v>
@@ -19698,8 +20010,10 @@
       <c r="L242" t="n">
         <v>4</v>
       </c>
-      <c r="M242" t="n">
-        <v>4</v>
+      <c r="M242" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N242" t="n">
         <v>1</v>
@@ -19777,8 +20091,10 @@
       <c r="L243" t="n">
         <v>4</v>
       </c>
-      <c r="M243" t="n">
-        <v>3</v>
+      <c r="M243" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="N243" t="n">
         <v>0</v>
@@ -19856,8 +20172,10 @@
       <c r="L244" t="n">
         <v>4</v>
       </c>
-      <c r="M244" t="n">
-        <v>1</v>
+      <c r="M244" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N244" t="n">
         <v>1</v>
@@ -20016,8 +20334,10 @@
       <c r="L246" t="n">
         <v>4</v>
       </c>
-      <c r="M246" t="n">
-        <v>4</v>
+      <c r="M246" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N246" t="n">
         <v>2</v>
@@ -20095,8 +20415,10 @@
       <c r="L247" t="n">
         <v>3</v>
       </c>
-      <c r="M247" t="n">
-        <v>5</v>
+      <c r="M247" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N247" t="n">
         <v>2</v>
@@ -20174,8 +20496,10 @@
       <c r="L248" t="n">
         <v>2</v>
       </c>
-      <c r="M248" t="n">
-        <v>4</v>
+      <c r="M248" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N248" t="n">
         <v>2</v>
@@ -20415,8 +20739,10 @@
       <c r="L251" t="n">
         <v>4</v>
       </c>
-      <c r="M251" t="n">
-        <v>4</v>
+      <c r="M251" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N251" t="n">
         <v>2</v>
@@ -20494,8 +20820,10 @@
       <c r="L252" t="n">
         <v>4</v>
       </c>
-      <c r="M252" t="n">
-        <v>4</v>
+      <c r="M252" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N252" t="n">
         <v>2</v>
@@ -20573,8 +20901,10 @@
       <c r="L253" t="n">
         <v>4</v>
       </c>
-      <c r="M253" t="n">
-        <v>4</v>
+      <c r="M253" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N253" t="n">
         <v>1</v>
@@ -20895,8 +21225,10 @@
       <c r="L257" t="n">
         <v>4</v>
       </c>
-      <c r="M257" t="n">
-        <v>5</v>
+      <c r="M257" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N257" t="n">
         <v>1</v>
@@ -20974,8 +21306,10 @@
       <c r="L258" t="n">
         <v>4</v>
       </c>
-      <c r="M258" t="n">
-        <v>5</v>
+      <c r="M258" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N258" t="n">
         <v>2</v>
@@ -21053,8 +21387,10 @@
       <c r="L259" t="n">
         <v>5</v>
       </c>
-      <c r="M259" t="n">
-        <v>4</v>
+      <c r="M259" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N259" t="n">
         <v>0</v>
@@ -21132,8 +21468,10 @@
       <c r="L260" t="n">
         <v>2</v>
       </c>
-      <c r="M260" t="n">
-        <v>4</v>
+      <c r="M260" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N260" t="n">
         <v>2</v>
@@ -21211,8 +21549,10 @@
       <c r="L261" t="n">
         <v>5</v>
       </c>
-      <c r="M261" t="n">
-        <v>1</v>
+      <c r="M261" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N261" t="n">
         <v>2</v>
@@ -21290,8 +21630,10 @@
       <c r="L262" t="n">
         <v>4</v>
       </c>
-      <c r="M262" t="n">
-        <v>1</v>
+      <c r="M262" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N262" t="n">
         <v>2</v>
@@ -21369,8 +21711,10 @@
       <c r="L263" t="n">
         <v>5</v>
       </c>
-      <c r="M263" t="n">
-        <v>1</v>
+      <c r="M263" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N263" t="n">
         <v>2</v>
@@ -21448,8 +21792,10 @@
       <c r="L264" t="n">
         <v>4</v>
       </c>
-      <c r="M264" t="n">
-        <v>4</v>
+      <c r="M264" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N264" t="n">
         <v>2</v>
@@ -21608,8 +21954,10 @@
       <c r="L266" t="n">
         <v>5</v>
       </c>
-      <c r="M266" t="n">
-        <v>5</v>
+      <c r="M266" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N266" t="n">
         <v>2</v>
@@ -21687,8 +22035,10 @@
       <c r="L267" t="n">
         <v>3</v>
       </c>
-      <c r="M267" t="n">
-        <v>4</v>
+      <c r="M267" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N267" t="n">
         <v>2</v>
@@ -21766,8 +22116,10 @@
       <c r="L268" t="n">
         <v>4</v>
       </c>
-      <c r="M268" t="n">
-        <v>2</v>
+      <c r="M268" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="N268" t="n">
         <v>2</v>
@@ -21845,8 +22197,10 @@
       <c r="L269" t="n">
         <v>4</v>
       </c>
-      <c r="M269" t="n">
-        <v>5</v>
+      <c r="M269" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N269" t="n">
         <v>2</v>
@@ -22005,8 +22359,10 @@
       <c r="L271" t="n">
         <v>5</v>
       </c>
-      <c r="M271" t="n">
-        <v>4</v>
+      <c r="M271" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N271" t="n">
         <v>2</v>
@@ -22084,8 +22440,10 @@
       <c r="L272" t="n">
         <v>5</v>
       </c>
-      <c r="M272" t="n">
-        <v>5</v>
+      <c r="M272" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N272" t="n">
         <v>2</v>
@@ -22163,8 +22521,10 @@
       <c r="L273" t="n">
         <v>4</v>
       </c>
-      <c r="M273" t="n">
-        <v>4</v>
+      <c r="M273" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N273" t="n">
         <v>2</v>
@@ -22323,8 +22683,10 @@
       <c r="L275" t="n">
         <v>4</v>
       </c>
-      <c r="M275" t="n">
-        <v>4</v>
+      <c r="M275" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N275" t="n">
         <v>2</v>
@@ -22402,8 +22764,10 @@
       <c r="L276" t="n">
         <v>4</v>
       </c>
-      <c r="M276" t="n">
-        <v>4</v>
+      <c r="M276" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N276" t="n">
         <v>2</v>
@@ -22481,8 +22845,10 @@
       <c r="L277" t="n">
         <v>5</v>
       </c>
-      <c r="M277" t="n">
-        <v>1</v>
+      <c r="M277" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N277" t="n">
         <v>2</v>
@@ -22560,8 +22926,10 @@
       <c r="L278" t="n">
         <v>4</v>
       </c>
-      <c r="M278" t="n">
-        <v>4</v>
+      <c r="M278" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N278" t="n">
         <v>2</v>
@@ -22639,8 +23007,10 @@
       <c r="L279" t="n">
         <v>4</v>
       </c>
-      <c r="M279" t="n">
-        <v>1</v>
+      <c r="M279" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N279" t="n">
         <v>1</v>
@@ -22718,8 +23088,10 @@
       <c r="L280" t="n">
         <v>4</v>
       </c>
-      <c r="M280" t="n">
-        <v>4</v>
+      <c r="M280" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N280" t="n">
         <v>2</v>
@@ -22797,8 +23169,10 @@
       <c r="L281" t="n">
         <v>4</v>
       </c>
-      <c r="M281" t="n">
-        <v>2</v>
+      <c r="M281" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="N281" t="n">
         <v>2</v>
@@ -22876,8 +23250,10 @@
       <c r="L282" t="n">
         <v>5</v>
       </c>
-      <c r="M282" t="n">
-        <v>1</v>
+      <c r="M282" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="N282" t="n">
         <v>2</v>
@@ -22955,8 +23331,10 @@
       <c r="L283" t="n">
         <v>4</v>
       </c>
-      <c r="M283" t="n">
-        <v>4</v>
+      <c r="M283" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N283" t="n">
         <v>2</v>
@@ -23034,8 +23412,10 @@
       <c r="L284" t="n">
         <v>4</v>
       </c>
-      <c r="M284" t="n">
-        <v>4</v>
+      <c r="M284" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N284" t="n">
         <v>1</v>
@@ -23113,8 +23493,10 @@
       <c r="L285" t="n">
         <v>2</v>
       </c>
-      <c r="M285" t="n">
-        <v>4</v>
+      <c r="M285" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N285" t="n">
         <v>2</v>
@@ -23192,8 +23574,10 @@
       <c r="L286" t="n">
         <v>3</v>
       </c>
-      <c r="M286" t="n">
-        <v>5</v>
+      <c r="M286" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="N286" t="n">
         <v>2</v>
@@ -23271,8 +23655,10 @@
       <c r="L287" t="n">
         <v>2</v>
       </c>
-      <c r="M287" t="n">
-        <v>4</v>
+      <c r="M287" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N287" t="n">
         <v>2</v>
@@ -23350,8 +23736,10 @@
       <c r="L288" t="n">
         <v>3</v>
       </c>
-      <c r="M288" t="n">
-        <v>4</v>
+      <c r="M288" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N288" t="n">
         <v>2</v>
@@ -23591,8 +23979,10 @@
       <c r="L291" t="n">
         <v>3</v>
       </c>
-      <c r="M291" t="n">
-        <v>4</v>
+      <c r="M291" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N291" t="n">
         <v>2</v>
@@ -23670,8 +24060,10 @@
       <c r="L292" t="n">
         <v>2</v>
       </c>
-      <c r="M292" t="n">
-        <v>4</v>
+      <c r="M292" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N292" t="n">
         <v>2</v>
@@ -23749,8 +24141,10 @@
       <c r="L293" t="n">
         <v>3</v>
       </c>
-      <c r="M293" t="n">
-        <v>4</v>
+      <c r="M293" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="N293" t="n">
         <v>2</v>

</xml_diff>